<commit_message>
Rev 4 - Laptop migration: new features + asset cleanup + tile pictures
</commit_message>
<xml_diff>
--- a/DATA/DATA FILES/GAS PACKS DATA.xlsx
+++ b/DATA/DATA FILES/GAS PACKS DATA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ericc\Documents\HHpro\DATA\DATA FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A1EC1D-6370-4C78-A8D8-8605B7DA86F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76AB235B-3AA4-4E55-BF06-EE429A861A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SCHEDULE" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2005" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="258">
   <si>
     <t>Fan Data</t>
   </si>
@@ -805,6 +805,9 @@
   </si>
   <si>
     <t>Provide with 24" factory roofcurb</t>
+  </si>
+  <si>
+    <t>OPERATION MANUAL</t>
   </si>
 </sst>
 </file>
@@ -1178,7 +1181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1324,8 +1327,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1386,9 +1389,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1773,7 +1773,7 @@
     <col min="46" max="46" width="14.5703125" style="21" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="14.5703125" style="21" customWidth="1"/>
     <col min="48" max="48" width="20" style="21" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="6.5703125" style="21" customWidth="1"/>
+    <col min="49" max="49" width="19.85546875" style="21" bestFit="1" customWidth="1"/>
     <col min="50" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -1830,8 +1830,8 @@
       <c r="AS1" s="53"/>
       <c r="AT1" s="53"/>
       <c r="AU1" s="53"/>
-      <c r="AV1" s="54"/>
-      <c r="AW1" s="45"/>
+      <c r="AV1" s="53"/>
+      <c r="AW1" s="54"/>
     </row>
     <row r="2" spans="1:49" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="61" t="s">
@@ -1929,7 +1929,9 @@
       <c r="AV2" s="50" t="s">
         <v>249</v>
       </c>
-      <c r="AW2" s="45"/>
+      <c r="AW2" s="50" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="3" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="64" t="s">
@@ -1997,7 +1999,7 @@
       <c r="AT3" s="51"/>
       <c r="AU3" s="51"/>
       <c r="AV3" s="51"/>
-      <c r="AW3" s="45"/>
+      <c r="AW3" s="51"/>
     </row>
     <row r="4" spans="1:49" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="65"/>
@@ -2083,7 +2085,7 @@
       <c r="AT4" s="51"/>
       <c r="AU4" s="51"/>
       <c r="AV4" s="51"/>
-      <c r="AW4" s="45"/>
+      <c r="AW4" s="51"/>
     </row>
     <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
@@ -2203,8 +2205,8 @@
       <c r="AU5" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="AV5" s="49"/>
-      <c r="AW5" s="46"/>
+      <c r="AV5" s="48"/>
+      <c r="AW5" s="26"/>
     </row>
     <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -2323,7 +2325,8 @@
       <c r="AU6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="AV6" s="28"/>
+      <c r="AV6" s="23"/>
+      <c r="AW6" s="28"/>
     </row>
     <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -2442,7 +2445,8 @@
       <c r="AU7" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="AV7" s="28"/>
+      <c r="AV7" s="23"/>
+      <c r="AW7" s="28"/>
     </row>
     <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
@@ -2561,7 +2565,8 @@
       <c r="AU8" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="AV8" s="28"/>
+      <c r="AV8" s="23"/>
+      <c r="AW8" s="28"/>
     </row>
     <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -2680,7 +2685,8 @@
       <c r="AU9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="AV9" s="28"/>
+      <c r="AV9" s="23"/>
+      <c r="AW9" s="28"/>
     </row>
     <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
@@ -2799,7 +2805,8 @@
       <c r="AU10" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AV10" s="28"/>
+      <c r="AV10" s="23"/>
+      <c r="AW10" s="28"/>
     </row>
     <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
@@ -2918,7 +2925,8 @@
       <c r="AU11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="AV11" s="28"/>
+      <c r="AV11" s="23"/>
+      <c r="AW11" s="28"/>
     </row>
     <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
@@ -3037,7 +3045,8 @@
       <c r="AU12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="AV12" s="28"/>
+      <c r="AV12" s="23"/>
+      <c r="AW12" s="28"/>
     </row>
     <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
@@ -3156,7 +3165,8 @@
       <c r="AU13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AV13" s="28"/>
+      <c r="AV13" s="23"/>
+      <c r="AW13" s="28"/>
     </row>
     <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
@@ -3275,7 +3285,8 @@
       <c r="AU14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="AV14" s="28"/>
+      <c r="AV14" s="23"/>
+      <c r="AW14" s="28"/>
     </row>
     <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
@@ -3394,7 +3405,8 @@
       <c r="AU15" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AV15" s="28"/>
+      <c r="AV15" s="23"/>
+      <c r="AW15" s="28"/>
     </row>
     <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
@@ -3513,9 +3525,10 @@
       <c r="AU16" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AV16" s="28"/>
+      <c r="AV16" s="23"/>
+      <c r="AW16" s="28"/>
     </row>
-    <row r="17" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>23</v>
       </c>
@@ -3632,9 +3645,10 @@
       <c r="AU17" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="AV17" s="28"/>
+      <c r="AV17" s="23"/>
+      <c r="AW17" s="28"/>
     </row>
-    <row r="18" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
@@ -3751,9 +3765,10 @@
       <c r="AU18" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="AV18" s="28"/>
+      <c r="AV18" s="23"/>
+      <c r="AW18" s="28"/>
     </row>
-    <row r="19" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
@@ -3870,9 +3885,10 @@
       <c r="AU19" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="AV19" s="28"/>
+      <c r="AV19" s="23"/>
+      <c r="AW19" s="28"/>
     </row>
-    <row r="20" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>23</v>
       </c>
@@ -3989,9 +4005,10 @@
       <c r="AU20" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="AV20" s="28"/>
+      <c r="AV20" s="23"/>
+      <c r="AW20" s="28"/>
     </row>
-    <row r="21" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -4108,9 +4125,10 @@
       <c r="AU21" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="AV21" s="28"/>
+      <c r="AV21" s="23"/>
+      <c r="AW21" s="28"/>
     </row>
-    <row r="22" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>23</v>
       </c>
@@ -4227,9 +4245,10 @@
       <c r="AU22" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="AV22" s="28"/>
+      <c r="AV22" s="23"/>
+      <c r="AW22" s="28"/>
     </row>
-    <row r="23" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
@@ -4346,9 +4365,10 @@
       <c r="AU23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AV23" s="28"/>
+      <c r="AV23" s="23"/>
+      <c r="AW23" s="28"/>
     </row>
-    <row r="24" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>23</v>
       </c>
@@ -4465,9 +4485,10 @@
       <c r="AU24" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AV24" s="28"/>
+      <c r="AV24" s="23"/>
+      <c r="AW24" s="28"/>
     </row>
-    <row r="25" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>23</v>
       </c>
@@ -4584,9 +4605,10 @@
       <c r="AU25" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AV25" s="28"/>
+      <c r="AV25" s="23"/>
+      <c r="AW25" s="28"/>
     </row>
-    <row r="26" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>23</v>
       </c>
@@ -4703,9 +4725,10 @@
       <c r="AU26" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="AV26" s="28"/>
+      <c r="AV26" s="23"/>
+      <c r="AW26" s="28"/>
     </row>
-    <row r="27" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>23</v>
       </c>
@@ -4822,9 +4845,10 @@
       <c r="AU27" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="AV27" s="28"/>
+      <c r="AV27" s="23"/>
+      <c r="AW27" s="28"/>
     </row>
-    <row r="28" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>23</v>
       </c>
@@ -4941,9 +4965,10 @@
       <c r="AU28" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="AV28" s="28"/>
+      <c r="AV28" s="23"/>
+      <c r="AW28" s="28"/>
     </row>
-    <row r="29" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>23</v>
       </c>
@@ -5060,9 +5085,10 @@
       <c r="AU29" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="AV29" s="28"/>
+      <c r="AV29" s="23"/>
+      <c r="AW29" s="28"/>
     </row>
-    <row r="30" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>23</v>
       </c>
@@ -5179,9 +5205,10 @@
       <c r="AU30" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="AV30" s="28"/>
+      <c r="AV30" s="23"/>
+      <c r="AW30" s="28"/>
     </row>
-    <row r="31" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>23</v>
       </c>
@@ -5298,9 +5325,10 @@
       <c r="AU31" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="AV31" s="28"/>
+      <c r="AV31" s="23"/>
+      <c r="AW31" s="28"/>
     </row>
-    <row r="32" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>23</v>
       </c>
@@ -5417,9 +5445,10 @@
       <c r="AU32" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="AV32" s="28"/>
+      <c r="AV32" s="23"/>
+      <c r="AW32" s="28"/>
     </row>
-    <row r="33" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>23</v>
       </c>
@@ -5536,9 +5565,10 @@
       <c r="AU33" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="AV33" s="28"/>
+      <c r="AV33" s="23"/>
+      <c r="AW33" s="28"/>
     </row>
-    <row r="34" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
@@ -5655,9 +5685,10 @@
       <c r="AU34" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="AV34" s="28"/>
+      <c r="AV34" s="23"/>
+      <c r="AW34" s="28"/>
     </row>
-    <row r="35" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>23</v>
       </c>
@@ -5774,9 +5805,10 @@
       <c r="AU35" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="AV35" s="28"/>
+      <c r="AV35" s="23"/>
+      <c r="AW35" s="28"/>
     </row>
-    <row r="36" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>23</v>
       </c>
@@ -5893,9 +5925,10 @@
       <c r="AU36" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="AV36" s="28"/>
+      <c r="AV36" s="23"/>
+      <c r="AW36" s="28"/>
     </row>
-    <row r="37" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>23</v>
       </c>
@@ -6012,9 +6045,10 @@
       <c r="AU37" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="AV37" s="28"/>
+      <c r="AV37" s="23"/>
+      <c r="AW37" s="28"/>
     </row>
-    <row r="38" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>23</v>
       </c>
@@ -6131,9 +6165,10 @@
       <c r="AU38" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AV38" s="28"/>
+      <c r="AV38" s="23"/>
+      <c r="AW38" s="28"/>
     </row>
-    <row r="39" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>23</v>
       </c>
@@ -6250,9 +6285,10 @@
       <c r="AU39" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="AV39" s="28"/>
+      <c r="AV39" s="23"/>
+      <c r="AW39" s="28"/>
     </row>
-    <row r="40" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>23</v>
       </c>
@@ -6369,9 +6405,10 @@
       <c r="AU40" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AV40" s="28"/>
+      <c r="AV40" s="23"/>
+      <c r="AW40" s="28"/>
     </row>
-    <row r="41" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>23</v>
       </c>
@@ -6488,9 +6525,10 @@
       <c r="AU41" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="AV41" s="28"/>
+      <c r="AV41" s="23"/>
+      <c r="AW41" s="28"/>
     </row>
-    <row r="42" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>23</v>
       </c>
@@ -6607,9 +6645,10 @@
       <c r="AU42" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="AV42" s="28"/>
+      <c r="AV42" s="23"/>
+      <c r="AW42" s="28"/>
     </row>
-    <row r="43" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>23</v>
       </c>
@@ -6726,9 +6765,10 @@
       <c r="AU43" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="AV43" s="28"/>
+      <c r="AV43" s="23"/>
+      <c r="AW43" s="28"/>
     </row>
-    <row r="44" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>23</v>
       </c>
@@ -6845,9 +6885,10 @@
       <c r="AU44" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="AV44" s="28"/>
+      <c r="AV44" s="23"/>
+      <c r="AW44" s="28"/>
     </row>
-    <row r="45" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>23</v>
       </c>
@@ -6964,9 +7005,10 @@
       <c r="AU45" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="AV45" s="28"/>
+      <c r="AV45" s="23"/>
+      <c r="AW45" s="28"/>
     </row>
-    <row r="46" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>23</v>
       </c>
@@ -7083,9 +7125,10 @@
       <c r="AU46" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="AV46" s="28"/>
+      <c r="AV46" s="23"/>
+      <c r="AW46" s="28"/>
     </row>
-    <row r="47" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>23</v>
       </c>
@@ -7202,9 +7245,10 @@
       <c r="AU47" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AV47" s="28"/>
+      <c r="AV47" s="23"/>
+      <c r="AW47" s="28"/>
     </row>
-    <row r="48" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>23</v>
       </c>
@@ -7321,9 +7365,10 @@
       <c r="AU48" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AV48" s="28"/>
+      <c r="AV48" s="23"/>
+      <c r="AW48" s="28"/>
     </row>
-    <row r="49" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>23</v>
       </c>
@@ -7440,9 +7485,10 @@
       <c r="AU49" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AV49" s="28"/>
+      <c r="AV49" s="23"/>
+      <c r="AW49" s="28"/>
     </row>
-    <row r="50" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>23</v>
       </c>
@@ -7559,9 +7605,10 @@
       <c r="AU50" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="AV50" s="28"/>
+      <c r="AV50" s="23"/>
+      <c r="AW50" s="28"/>
     </row>
-    <row r="51" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>23</v>
       </c>
@@ -7678,9 +7725,10 @@
       <c r="AU51" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AV51" s="28"/>
+      <c r="AV51" s="23"/>
+      <c r="AW51" s="28"/>
     </row>
-    <row r="52" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>23</v>
       </c>
@@ -7797,9 +7845,10 @@
       <c r="AU52" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="AV52" s="28"/>
+      <c r="AV52" s="23"/>
+      <c r="AW52" s="28"/>
     </row>
-    <row r="53" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>23</v>
       </c>
@@ -7916,9 +7965,10 @@
       <c r="AU53" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="AV53" s="28"/>
+      <c r="AV53" s="23"/>
+      <c r="AW53" s="28"/>
     </row>
-    <row r="54" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>23</v>
       </c>
@@ -8035,9 +8085,10 @@
       <c r="AU54" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="AV54" s="28"/>
+      <c r="AV54" s="23"/>
+      <c r="AW54" s="28"/>
     </row>
-    <row r="55" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>23</v>
       </c>
@@ -8154,9 +8205,10 @@
       <c r="AU55" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AV55" s="28"/>
+      <c r="AV55" s="23"/>
+      <c r="AW55" s="28"/>
     </row>
-    <row r="56" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>23</v>
       </c>
@@ -8273,9 +8325,10 @@
       <c r="AU56" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="AV56" s="28"/>
+      <c r="AV56" s="23"/>
+      <c r="AW56" s="28"/>
     </row>
-    <row r="57" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>23</v>
       </c>
@@ -8392,9 +8445,10 @@
       <c r="AU57" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="AV57" s="28"/>
+      <c r="AV57" s="23"/>
+      <c r="AW57" s="28"/>
     </row>
-    <row r="58" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>23</v>
       </c>
@@ -8511,9 +8565,10 @@
       <c r="AU58" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="AV58" s="28"/>
+      <c r="AV58" s="23"/>
+      <c r="AW58" s="28"/>
     </row>
-    <row r="59" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>23</v>
       </c>
@@ -8630,9 +8685,10 @@
       <c r="AU59" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AV59" s="28"/>
+      <c r="AV59" s="23"/>
+      <c r="AW59" s="28"/>
     </row>
-    <row r="60" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>23</v>
       </c>
@@ -8749,9 +8805,10 @@
       <c r="AU60" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="AV60" s="28"/>
+      <c r="AV60" s="23"/>
+      <c r="AW60" s="28"/>
     </row>
-    <row r="61" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>23</v>
       </c>
@@ -8868,9 +8925,10 @@
       <c r="AU61" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="AV61" s="28"/>
+      <c r="AV61" s="23"/>
+      <c r="AW61" s="28"/>
     </row>
-    <row r="62" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>23</v>
       </c>
@@ -8987,9 +9045,10 @@
       <c r="AU62" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AV62" s="28"/>
+      <c r="AV62" s="23"/>
+      <c r="AW62" s="28"/>
     </row>
-    <row r="63" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>23</v>
       </c>
@@ -9106,9 +9165,10 @@
       <c r="AU63" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AV63" s="28"/>
+      <c r="AV63" s="23"/>
+      <c r="AW63" s="28"/>
     </row>
-    <row r="64" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>23</v>
       </c>
@@ -9225,9 +9285,10 @@
       <c r="AU64" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AV64" s="28"/>
+      <c r="AV64" s="23"/>
+      <c r="AW64" s="28"/>
     </row>
-    <row r="65" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>23</v>
       </c>
@@ -9344,9 +9405,10 @@
       <c r="AU65" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="AV65" s="28"/>
+      <c r="AV65" s="23"/>
+      <c r="AW65" s="28"/>
     </row>
-    <row r="66" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>23</v>
       </c>
@@ -9463,9 +9525,10 @@
       <c r="AU66" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="AV66" s="28"/>
+      <c r="AV66" s="23"/>
+      <c r="AW66" s="28"/>
     </row>
-    <row r="67" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>23</v>
       </c>
@@ -9582,9 +9645,10 @@
       <c r="AU67" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="AV67" s="28"/>
+      <c r="AV67" s="23"/>
+      <c r="AW67" s="28"/>
     </row>
-    <row r="68" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>23</v>
       </c>
@@ -9701,9 +9765,10 @@
       <c r="AU68" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="AV68" s="28"/>
+      <c r="AV68" s="23"/>
+      <c r="AW68" s="28"/>
     </row>
-    <row r="69" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>23</v>
       </c>
@@ -9820,9 +9885,10 @@
       <c r="AU69" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="AV69" s="28"/>
+      <c r="AV69" s="23"/>
+      <c r="AW69" s="28"/>
     </row>
-    <row r="70" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>23</v>
       </c>
@@ -9939,9 +10005,10 @@
       <c r="AU70" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="AV70" s="28"/>
+      <c r="AV70" s="23"/>
+      <c r="AW70" s="28"/>
     </row>
-    <row r="71" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>23</v>
       </c>
@@ -10058,9 +10125,10 @@
       <c r="AU71" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="AV71" s="28"/>
+      <c r="AV71" s="23"/>
+      <c r="AW71" s="28"/>
     </row>
-    <row r="72" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>23</v>
       </c>
@@ -10177,9 +10245,10 @@
       <c r="AU72" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="AV72" s="28"/>
+      <c r="AV72" s="23"/>
+      <c r="AW72" s="28"/>
     </row>
-    <row r="73" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>23</v>
       </c>
@@ -10296,9 +10365,10 @@
       <c r="AU73" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="AV73" s="28"/>
+      <c r="AV73" s="23"/>
+      <c r="AW73" s="28"/>
     </row>
-    <row r="74" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>23</v>
       </c>
@@ -10415,9 +10485,10 @@
       <c r="AU74" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="AV74" s="28"/>
+      <c r="AV74" s="23"/>
+      <c r="AW74" s="28"/>
     </row>
-    <row r="75" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
         <v>23</v>
       </c>
@@ -10534,9 +10605,10 @@
       <c r="AU75" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="AV75" s="28"/>
+      <c r="AV75" s="23"/>
+      <c r="AW75" s="28"/>
     </row>
-    <row r="76" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>23</v>
       </c>
@@ -10653,9 +10725,10 @@
       <c r="AU76" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="AV76" s="28"/>
+      <c r="AV76" s="23"/>
+      <c r="AW76" s="28"/>
     </row>
-    <row r="77" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>23</v>
       </c>
@@ -10772,9 +10845,10 @@
       <c r="AU77" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="AV77" s="28"/>
+      <c r="AV77" s="23"/>
+      <c r="AW77" s="28"/>
     </row>
-    <row r="78" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>23</v>
       </c>
@@ -10891,9 +10965,10 @@
       <c r="AU78" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="AV78" s="28"/>
+      <c r="AV78" s="23"/>
+      <c r="AW78" s="28"/>
     </row>
-    <row r="79" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>23</v>
       </c>
@@ -11010,9 +11085,10 @@
       <c r="AU79" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="AV79" s="28"/>
+      <c r="AV79" s="23"/>
+      <c r="AW79" s="28"/>
     </row>
-    <row r="80" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>23</v>
       </c>
@@ -11129,9 +11205,10 @@
       <c r="AU80" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="AV80" s="28"/>
+      <c r="AV80" s="23"/>
+      <c r="AW80" s="28"/>
     </row>
-    <row r="81" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>23</v>
       </c>
@@ -11248,9 +11325,10 @@
       <c r="AU81" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="AV81" s="28"/>
+      <c r="AV81" s="23"/>
+      <c r="AW81" s="28"/>
     </row>
-    <row r="82" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>23</v>
       </c>
@@ -11367,9 +11445,10 @@
       <c r="AU82" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="AV82" s="28"/>
+      <c r="AV82" s="23"/>
+      <c r="AW82" s="28"/>
     </row>
-    <row r="83" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>23</v>
       </c>
@@ -11486,9 +11565,10 @@
       <c r="AU83" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="AV83" s="28"/>
+      <c r="AV83" s="23"/>
+      <c r="AW83" s="28"/>
     </row>
-    <row r="84" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
         <v>23</v>
       </c>
@@ -11605,9 +11685,10 @@
       <c r="AU84" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="AV84" s="28"/>
+      <c r="AV84" s="23"/>
+      <c r="AW84" s="28"/>
     </row>
-    <row r="85" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>23</v>
       </c>
@@ -11724,9 +11805,10 @@
       <c r="AU85" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="AV85" s="28"/>
+      <c r="AV85" s="23"/>
+      <c r="AW85" s="28"/>
     </row>
-    <row r="86" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>23</v>
       </c>
@@ -11843,9 +11925,10 @@
       <c r="AU86" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="AV86" s="28"/>
+      <c r="AV86" s="23"/>
+      <c r="AW86" s="28"/>
     </row>
-    <row r="87" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
         <v>23</v>
       </c>
@@ -11962,9 +12045,10 @@
       <c r="AU87" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="AV87" s="28"/>
+      <c r="AV87" s="23"/>
+      <c r="AW87" s="28"/>
     </row>
-    <row r="88" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>23</v>
       </c>
@@ -12081,9 +12165,10 @@
       <c r="AU88" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="AV88" s="28"/>
+      <c r="AV88" s="23"/>
+      <c r="AW88" s="28"/>
     </row>
-    <row r="89" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>23</v>
       </c>
@@ -12200,9 +12285,10 @@
       <c r="AU89" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="AV89" s="28"/>
+      <c r="AV89" s="23"/>
+      <c r="AW89" s="28"/>
     </row>
-    <row r="90" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
         <v>23</v>
       </c>
@@ -12319,9 +12405,10 @@
       <c r="AU90" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="AV90" s="28"/>
+      <c r="AV90" s="23"/>
+      <c r="AW90" s="28"/>
     </row>
-    <row r="91" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
         <v>23</v>
       </c>
@@ -12438,9 +12525,10 @@
       <c r="AU91" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="AV91" s="28"/>
+      <c r="AV91" s="23"/>
+      <c r="AW91" s="28"/>
     </row>
-    <row r="92" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
         <v>23</v>
       </c>
@@ -12557,9 +12645,10 @@
       <c r="AU92" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="AV92" s="28"/>
+      <c r="AV92" s="23"/>
+      <c r="AW92" s="28"/>
     </row>
-    <row r="93" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
         <v>23</v>
       </c>
@@ -12676,9 +12765,10 @@
       <c r="AU93" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="AV93" s="28"/>
+      <c r="AV93" s="23"/>
+      <c r="AW93" s="28"/>
     </row>
-    <row r="94" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>23</v>
       </c>
@@ -12795,9 +12885,10 @@
       <c r="AU94" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="AV94" s="28"/>
+      <c r="AV94" s="23"/>
+      <c r="AW94" s="28"/>
     </row>
-    <row r="95" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>23</v>
       </c>
@@ -12914,9 +13005,10 @@
       <c r="AU95" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="AV95" s="28"/>
+      <c r="AV95" s="23"/>
+      <c r="AW95" s="28"/>
     </row>
-    <row r="96" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
         <v>23</v>
       </c>
@@ -13033,9 +13125,10 @@
       <c r="AU96" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="AV96" s="28"/>
+      <c r="AV96" s="23"/>
+      <c r="AW96" s="28"/>
     </row>
-    <row r="97" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>23</v>
       </c>
@@ -13152,9 +13245,10 @@
       <c r="AU97" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="AV97" s="28"/>
+      <c r="AV97" s="23"/>
+      <c r="AW97" s="28"/>
     </row>
-    <row r="98" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>23</v>
       </c>
@@ -13271,9 +13365,10 @@
       <c r="AU98" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="AV98" s="28"/>
+      <c r="AV98" s="23"/>
+      <c r="AW98" s="28"/>
     </row>
-    <row r="99" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
         <v>23</v>
       </c>
@@ -13390,9 +13485,10 @@
       <c r="AU99" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="AV99" s="28"/>
+      <c r="AV99" s="23"/>
+      <c r="AW99" s="28"/>
     </row>
-    <row r="100" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>23</v>
       </c>
@@ -13509,9 +13605,10 @@
       <c r="AU100" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="AV100" s="28"/>
+      <c r="AV100" s="23"/>
+      <c r="AW100" s="28"/>
     </row>
-    <row r="101" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
         <v>23</v>
       </c>
@@ -13628,9 +13725,10 @@
       <c r="AU101" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="AV101" s="28"/>
+      <c r="AV101" s="23"/>
+      <c r="AW101" s="28"/>
     </row>
-    <row r="102" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>23</v>
       </c>
@@ -13747,9 +13845,10 @@
       <c r="AU102" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="AV102" s="28"/>
+      <c r="AV102" s="23"/>
+      <c r="AW102" s="28"/>
     </row>
-    <row r="103" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
         <v>23</v>
       </c>
@@ -13866,9 +13965,10 @@
       <c r="AU103" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="AV103" s="28"/>
+      <c r="AV103" s="23"/>
+      <c r="AW103" s="28"/>
     </row>
-    <row r="104" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>23</v>
       </c>
@@ -13985,9 +14085,10 @@
       <c r="AU104" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="AV104" s="28"/>
+      <c r="AV104" s="23"/>
+      <c r="AW104" s="28"/>
     </row>
-    <row r="105" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>23</v>
       </c>
@@ -14104,9 +14205,10 @@
       <c r="AU105" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="AV105" s="28"/>
+      <c r="AV105" s="23"/>
+      <c r="AW105" s="28"/>
     </row>
-    <row r="106" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
         <v>23</v>
       </c>
@@ -14223,9 +14325,10 @@
       <c r="AU106" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="AV106" s="28"/>
+      <c r="AV106" s="23"/>
+      <c r="AW106" s="28"/>
     </row>
-    <row r="107" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
         <v>23</v>
       </c>
@@ -14342,9 +14445,10 @@
       <c r="AU107" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="AV107" s="28"/>
+      <c r="AV107" s="23"/>
+      <c r="AW107" s="28"/>
     </row>
-    <row r="108" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
         <v>23</v>
       </c>
@@ -14461,9 +14565,10 @@
       <c r="AU108" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="AV108" s="28"/>
+      <c r="AV108" s="23"/>
+      <c r="AW108" s="28"/>
     </row>
-    <row r="109" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
         <v>23</v>
       </c>
@@ -14580,9 +14685,10 @@
       <c r="AU109" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="AV109" s="28"/>
+      <c r="AV109" s="23"/>
+      <c r="AW109" s="28"/>
     </row>
-    <row r="110" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A110" s="5" t="s">
         <v>23</v>
       </c>
@@ -14699,9 +14805,10 @@
       <c r="AU110" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="AV110" s="28"/>
+      <c r="AV110" s="23"/>
+      <c r="AW110" s="28"/>
     </row>
-    <row r="111" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A111" s="5" t="s">
         <v>23</v>
       </c>
@@ -14818,9 +14925,10 @@
       <c r="AU111" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="AV111" s="28"/>
+      <c r="AV111" s="23"/>
+      <c r="AW111" s="28"/>
     </row>
-    <row r="112" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A112" s="5" t="s">
         <v>23</v>
       </c>
@@ -14937,9 +15045,10 @@
       <c r="AU112" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="AV112" s="28"/>
+      <c r="AV112" s="23"/>
+      <c r="AW112" s="28"/>
     </row>
-    <row r="113" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A113" s="5" t="s">
         <v>23</v>
       </c>
@@ -15056,9 +15165,10 @@
       <c r="AU113" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="AV113" s="28"/>
+      <c r="AV113" s="23"/>
+      <c r="AW113" s="28"/>
     </row>
-    <row r="114" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A114" s="5" t="s">
         <v>23</v>
       </c>
@@ -15175,9 +15285,10 @@
       <c r="AU114" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="AV114" s="28"/>
+      <c r="AV114" s="23"/>
+      <c r="AW114" s="28"/>
     </row>
-    <row r="115" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A115" s="5" t="s">
         <v>23</v>
       </c>
@@ -15294,9 +15405,10 @@
       <c r="AU115" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="AV115" s="28"/>
+      <c r="AV115" s="23"/>
+      <c r="AW115" s="28"/>
     </row>
-    <row r="116" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A116" s="5" t="s">
         <v>23</v>
       </c>
@@ -15413,9 +15525,10 @@
       <c r="AU116" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="AV116" s="28"/>
+      <c r="AV116" s="23"/>
+      <c r="AW116" s="28"/>
     </row>
-    <row r="117" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A117" s="5" t="s">
         <v>23</v>
       </c>
@@ -15532,9 +15645,10 @@
       <c r="AU117" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="AV117" s="28"/>
+      <c r="AV117" s="23"/>
+      <c r="AW117" s="28"/>
     </row>
-    <row r="118" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A118" s="5" t="s">
         <v>23</v>
       </c>
@@ -15651,9 +15765,10 @@
       <c r="AU118" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="AV118" s="28"/>
+      <c r="AV118" s="23"/>
+      <c r="AW118" s="28"/>
     </row>
-    <row r="119" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A119" s="11" t="s">
         <v>23</v>
       </c>
@@ -15770,9 +15885,10 @@
       <c r="AU119" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="AV119" s="28"/>
+      <c r="AV119" s="23"/>
+      <c r="AW119" s="28"/>
     </row>
-    <row r="120" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A120" s="11" t="s">
         <v>23</v>
       </c>
@@ -15889,9 +16005,10 @@
       <c r="AU120" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="AV120" s="28"/>
+      <c r="AV120" s="23"/>
+      <c r="AW120" s="28"/>
     </row>
-    <row r="121" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A121" s="11" t="s">
         <v>23</v>
       </c>
@@ -16008,9 +16125,10 @@
       <c r="AU121" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="AV121" s="28"/>
+      <c r="AV121" s="23"/>
+      <c r="AW121" s="28"/>
     </row>
-    <row r="122" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A122" s="11" t="s">
         <v>23</v>
       </c>
@@ -16127,9 +16245,10 @@
       <c r="AU122" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="AV122" s="28"/>
+      <c r="AV122" s="23"/>
+      <c r="AW122" s="28"/>
     </row>
-    <row r="123" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A123" s="11" t="s">
         <v>23</v>
       </c>
@@ -16246,9 +16365,10 @@
       <c r="AU123" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AV123" s="28"/>
+      <c r="AV123" s="23"/>
+      <c r="AW123" s="28"/>
     </row>
-    <row r="124" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A124" s="11" t="s">
         <v>23</v>
       </c>
@@ -16365,9 +16485,10 @@
       <c r="AU124" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="AV124" s="28"/>
+      <c r="AV124" s="23"/>
+      <c r="AW124" s="28"/>
     </row>
-    <row r="125" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A125" s="11" t="s">
         <v>23</v>
       </c>
@@ -16484,9 +16605,10 @@
       <c r="AU125" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AV125" s="28"/>
+      <c r="AV125" s="23"/>
+      <c r="AW125" s="28"/>
     </row>
-    <row r="126" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A126" s="11" t="s">
         <v>23</v>
       </c>
@@ -16603,9 +16725,10 @@
       <c r="AU126" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AV126" s="28"/>
+      <c r="AV126" s="23"/>
+      <c r="AW126" s="28"/>
     </row>
-    <row r="127" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A127" s="11" t="s">
         <v>23</v>
       </c>
@@ -16722,9 +16845,10 @@
       <c r="AU127" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="AV127" s="28"/>
+      <c r="AV127" s="23"/>
+      <c r="AW127" s="28"/>
     </row>
-    <row r="128" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A128" s="11" t="s">
         <v>23</v>
       </c>
@@ -16841,9 +16965,10 @@
       <c r="AU128" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="AV128" s="28"/>
+      <c r="AV128" s="23"/>
+      <c r="AW128" s="28"/>
     </row>
-    <row r="129" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A129" s="11" t="s">
         <v>23</v>
       </c>
@@ -16960,9 +17085,10 @@
       <c r="AU129" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="AV129" s="28"/>
+      <c r="AV129" s="23"/>
+      <c r="AW129" s="28"/>
     </row>
-    <row r="130" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>23</v>
       </c>
@@ -17079,9 +17205,10 @@
       <c r="AU130" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="AV130" s="28"/>
+      <c r="AV130" s="23"/>
+      <c r="AW130" s="28"/>
     </row>
-    <row r="131" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A131" s="11" t="s">
         <v>23</v>
       </c>
@@ -17198,9 +17325,10 @@
       <c r="AU131" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="AV131" s="28"/>
+      <c r="AV131" s="23"/>
+      <c r="AW131" s="28"/>
     </row>
-    <row r="132" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A132" s="11" t="s">
         <v>23</v>
       </c>
@@ -17317,9 +17445,10 @@
       <c r="AU132" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="AV132" s="28"/>
+      <c r="AV132" s="23"/>
+      <c r="AW132" s="28"/>
     </row>
-    <row r="133" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A133" s="11" t="s">
         <v>23</v>
       </c>
@@ -17436,9 +17565,10 @@
       <c r="AU133" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="AV133" s="28"/>
+      <c r="AV133" s="23"/>
+      <c r="AW133" s="28"/>
     </row>
-    <row r="134" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A134" s="11" t="s">
         <v>23</v>
       </c>
@@ -17555,9 +17685,10 @@
       <c r="AU134" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="AV134" s="28"/>
+      <c r="AV134" s="23"/>
+      <c r="AW134" s="28"/>
     </row>
-    <row r="135" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A135" s="11" t="s">
         <v>23</v>
       </c>
@@ -17674,9 +17805,10 @@
       <c r="AU135" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="AV135" s="28"/>
+      <c r="AV135" s="23"/>
+      <c r="AW135" s="28"/>
     </row>
-    <row r="136" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A136" s="11" t="s">
         <v>23</v>
       </c>
@@ -17793,9 +17925,10 @@
       <c r="AU136" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="AV136" s="28"/>
+      <c r="AV136" s="23"/>
+      <c r="AW136" s="28"/>
     </row>
-    <row r="137" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A137" s="11" t="s">
         <v>23</v>
       </c>
@@ -17912,9 +18045,10 @@
       <c r="AU137" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="AV137" s="28"/>
+      <c r="AV137" s="23"/>
+      <c r="AW137" s="28"/>
     </row>
-    <row r="138" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A138" s="11" t="s">
         <v>23</v>
       </c>
@@ -18031,9 +18165,10 @@
       <c r="AU138" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="AV138" s="28"/>
+      <c r="AV138" s="23"/>
+      <c r="AW138" s="28"/>
     </row>
-    <row r="139" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A139" s="11" t="s">
         <v>23</v>
       </c>
@@ -18150,9 +18285,10 @@
       <c r="AU139" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="AV139" s="28"/>
+      <c r="AV139" s="23"/>
+      <c r="AW139" s="28"/>
     </row>
-    <row r="140" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A140" s="11" t="s">
         <v>23</v>
       </c>
@@ -18269,9 +18405,10 @@
       <c r="AU140" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="AV140" s="28"/>
+      <c r="AV140" s="23"/>
+      <c r="AW140" s="28"/>
     </row>
-    <row r="141" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A141" s="11" t="s">
         <v>23</v>
       </c>
@@ -18388,9 +18525,10 @@
       <c r="AU141" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="AV141" s="28"/>
+      <c r="AV141" s="23"/>
+      <c r="AW141" s="28"/>
     </row>
-    <row r="142" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A142" s="11" t="s">
         <v>23</v>
       </c>
@@ -18507,9 +18645,10 @@
       <c r="AU142" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="AV142" s="28"/>
+      <c r="AV142" s="23"/>
+      <c r="AW142" s="28"/>
     </row>
-    <row r="143" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A143" s="11" t="s">
         <v>23</v>
       </c>
@@ -18626,9 +18765,10 @@
       <c r="AU143" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AV143" s="28"/>
+      <c r="AV143" s="23"/>
+      <c r="AW143" s="28"/>
     </row>
-    <row r="144" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A144" s="11" t="s">
         <v>23</v>
       </c>
@@ -18745,9 +18885,10 @@
       <c r="AU144" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="AV144" s="28"/>
+      <c r="AV144" s="23"/>
+      <c r="AW144" s="28"/>
     </row>
-    <row r="145" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A145" s="11" t="s">
         <v>23</v>
       </c>
@@ -18864,9 +19005,10 @@
       <c r="AU145" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="AV145" s="28"/>
+      <c r="AV145" s="23"/>
+      <c r="AW145" s="28"/>
     </row>
-    <row r="146" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A146" s="11" t="s">
         <v>23</v>
       </c>
@@ -18983,9 +19125,10 @@
       <c r="AU146" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="AV146" s="28"/>
+      <c r="AV146" s="23"/>
+      <c r="AW146" s="28"/>
     </row>
-    <row r="147" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A147" s="11" t="s">
         <v>23</v>
       </c>
@@ -19102,9 +19245,10 @@
       <c r="AU147" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AV147" s="28"/>
+      <c r="AV147" s="23"/>
+      <c r="AW147" s="28"/>
     </row>
-    <row r="148" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A148" s="11" t="s">
         <v>23</v>
       </c>
@@ -19221,9 +19365,10 @@
       <c r="AU148" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="AV148" s="28"/>
+      <c r="AV148" s="23"/>
+      <c r="AW148" s="28"/>
     </row>
-    <row r="149" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A149" s="11" t="s">
         <v>23</v>
       </c>
@@ -19340,9 +19485,10 @@
       <c r="AU149" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="AV149" s="28"/>
+      <c r="AV149" s="23"/>
+      <c r="AW149" s="28"/>
     </row>
-    <row r="150" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A150" s="11" t="s">
         <v>23</v>
       </c>
@@ -19459,9 +19605,10 @@
       <c r="AU150" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="AV150" s="28"/>
+      <c r="AV150" s="23"/>
+      <c r="AW150" s="28"/>
     </row>
-    <row r="151" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A151" s="11" t="s">
         <v>23</v>
       </c>
@@ -19578,9 +19725,10 @@
       <c r="AU151" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="AV151" s="28"/>
+      <c r="AV151" s="23"/>
+      <c r="AW151" s="28"/>
     </row>
-    <row r="152" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A152" s="11" t="s">
         <v>23</v>
       </c>
@@ -19697,9 +19845,10 @@
       <c r="AU152" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="AV152" s="28"/>
+      <c r="AV152" s="23"/>
+      <c r="AW152" s="28"/>
     </row>
-    <row r="153" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
         <v>23</v>
       </c>
@@ -19816,9 +19965,10 @@
       <c r="AU153" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="AV153" s="28"/>
+      <c r="AV153" s="23"/>
+      <c r="AW153" s="28"/>
     </row>
-    <row r="154" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
         <v>23</v>
       </c>
@@ -19935,9 +20085,10 @@
       <c r="AU154" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="AV154" s="28"/>
+      <c r="AV154" s="23"/>
+      <c r="AW154" s="28"/>
     </row>
-    <row r="155" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
         <v>23</v>
       </c>
@@ -20054,9 +20205,10 @@
       <c r="AU155" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="AV155" s="28"/>
+      <c r="AV155" s="23"/>
+      <c r="AW155" s="28"/>
     </row>
-    <row r="156" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
         <v>23</v>
       </c>
@@ -20173,9 +20325,10 @@
       <c r="AU156" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="AV156" s="28"/>
+      <c r="AV156" s="23"/>
+      <c r="AW156" s="28"/>
     </row>
-    <row r="157" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
         <v>23</v>
       </c>
@@ -20292,9 +20445,10 @@
       <c r="AU157" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="AV157" s="28"/>
+      <c r="AV157" s="23"/>
+      <c r="AW157" s="28"/>
     </row>
-    <row r="158" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
         <v>23</v>
       </c>
@@ -20411,9 +20565,10 @@
       <c r="AU158" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="AV158" s="28"/>
+      <c r="AV158" s="23"/>
+      <c r="AW158" s="28"/>
     </row>
-    <row r="159" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
         <v>23</v>
       </c>
@@ -20530,9 +20685,10 @@
       <c r="AU159" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="AV159" s="28"/>
+      <c r="AV159" s="23"/>
+      <c r="AW159" s="28"/>
     </row>
-    <row r="160" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
         <v>23</v>
       </c>
@@ -20649,9 +20805,10 @@
       <c r="AU160" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="AV160" s="28"/>
+      <c r="AV160" s="23"/>
+      <c r="AW160" s="28"/>
     </row>
-    <row r="161" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
         <v>23</v>
       </c>
@@ -20768,9 +20925,10 @@
       <c r="AU161" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="AV161" s="28"/>
+      <c r="AV161" s="23"/>
+      <c r="AW161" s="28"/>
     </row>
-    <row r="162" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
         <v>23</v>
       </c>
@@ -20887,9 +21045,10 @@
       <c r="AU162" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="AV162" s="28"/>
+      <c r="AV162" s="23"/>
+      <c r="AW162" s="28"/>
     </row>
-    <row r="163" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
         <v>23</v>
       </c>
@@ -21006,9 +21165,10 @@
       <c r="AU163" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="AV163" s="28"/>
+      <c r="AV163" s="23"/>
+      <c r="AW163" s="28"/>
     </row>
-    <row r="164" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
         <v>23</v>
       </c>
@@ -21125,9 +21285,10 @@
       <c r="AU164" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="AV164" s="28"/>
+      <c r="AV164" s="23"/>
+      <c r="AW164" s="28"/>
     </row>
-    <row r="165" spans="1:48" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
         <v>23</v>
       </c>
@@ -21244,9 +21405,10 @@
       <c r="AU165" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="AV165" s="28"/>
+      <c r="AV165" s="23"/>
+      <c r="AW165" s="28"/>
     </row>
-    <row r="166" spans="1:48" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:49" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A166" s="12" t="s">
         <v>23</v>
       </c>
@@ -21363,15 +21525,17 @@
       <c r="AU166" s="42" t="s">
         <v>140</v>
       </c>
-      <c r="AV166" s="31"/>
+      <c r="AV166" s="30"/>
+      <c r="AW166" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="D3:F3"/>
+  <mergeCells count="37">
+    <mergeCell ref="AF1:AW1"/>
     <mergeCell ref="G3:M3"/>
     <mergeCell ref="N3:Q3"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="AH2:AH4"/>
+    <mergeCell ref="AW2:AW4"/>
     <mergeCell ref="AO2:AO4"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="Y1:AD1"/>
@@ -21387,9 +21551,9 @@
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="T3:W3"/>
+    <mergeCell ref="D3:F3"/>
     <mergeCell ref="AR2:AR4"/>
     <mergeCell ref="AU2:AU4"/>
-    <mergeCell ref="AF1:AV1"/>
     <mergeCell ref="AF2:AF4"/>
     <mergeCell ref="AG2:AG4"/>
     <mergeCell ref="AI2:AI4"/>
@@ -21414,37 +21578,37 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="49" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="49" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="70" t="s">
+      <c r="A3" s="49" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="70" t="s">
+      <c r="A4" s="49" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="70" t="s">
+      <c r="A5" s="49" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="70" t="s">
+      <c r="A6" s="49" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="49" t="s">
         <v>256</v>
       </c>
     </row>

</xml_diff>